<commit_message>
feat(curriculum): integrate Automatic Addison video series and report templates for Week 1, 2, and 3
</commit_message>
<xml_diff>
--- a/Apex_Autonomous_7Week_Plan.xlsx
+++ b/Apex_Autonomous_7Week_Plan.xlsx
@@ -1190,8 +1190,10 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>• ROS 2 Basics &amp; Nodes (Articulated Robotics): https://www.youtube.com/watch?v=0aPbWsyS3j0
-• ROS 2 Computational Graph: https://www.youtube.com/watch?v=1F_s5w2_6E4</t>
+          <t>• Package Guide: https://www.youtube.com/watch?v=DM77KkIJsik&amp;list=PLNWNEEf8BvG64FVZT4IdieI1PuYnHkUrt
+• ROS 2 Pub (Python): https://www.youtube.com/watch?v=jsVEhmXSTgc&amp;list=PLNWNEEf8BvG64FVZT4IdieI1PuYnHkUrt&amp;index=2
+• ROS 2 Sub (Python): https://youtube.com/playlist?list=PLNWNEEf8BvG64FVZT4IdieI1PuYnHkUrt&amp;si=Hk0_bWK0R5Ulyd_r
+• C++ Pub/Sub: https://youtu.be/EGLLMJPkzUQ | https://youtu.be/jABgxqDxcMA</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1250,7 +1252,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>• ROS 2 Pub/Sub in Python (Robotics Back-End): https://www.youtube.com/watch?v=cM_63A5o1-4</t>
+          <t>• ROS 2 Pub/Sub in Python (Automatic Addison): https://www.youtube.com/watch?v=jsVEhmXSTgc</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1309,7 +1311,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>• ROS 2 Launch Files in Python: https://www.youtube.com/watch?v=H7435f49uXg
+          <t>• ROS 2 Launch Files: https://youtu.be/2ri0Ouc67W0
 • rqt_graph Guide: https://docs.ros.org/en/humble/Tutorials/Beginner-CLI-Tools/Understanding-ROS2-Topics.html</t>
         </is>
       </c>
@@ -1461,8 +1463,10 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>• Building Robot with URDF &amp; Xacro: https://www.youtube.com/watch?v=BmjPA8W81Y0
-• REP-105 Standard: https://www.ros.org/reps/rep-0105.html</t>
+          <t>• Coordinate Frames: https://youtu.be/oxr8df96tWk
+• Mobile Robot URDF: https://youtu.be/XtS8mCcffrs
+• URDF Launch Files: https://youtu.be/2ri0Ouc67W0
+• RViz Parameters: https://youtu.be/AkekfmNAUkk</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1490,7 +1494,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>• RViz2 Beginner Tutorial: https://www.youtube.com/watch?v=1-3mZ4A9Tlg</t>
+          <t>• RViz Parameters Guide: https://youtu.be/AkekfmNAUkk</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -1519,7 +1523,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>• URDF Wheel Joints &amp; Wheels: https://www.youtube.com/watch?v=e4B2jLh8ZkY</t>
+          <t>• Mobile Robot URDF (Automatic Addison): https://youtu.be/XtS8mCcffrs</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1548,7 +1552,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>• Understanding TF Tree (Articulated Robotics): https://www.youtube.com/watch?v=Qyv4GZp4UGE</t>
+          <t>• Coordinate Frame Basics: https://youtu.be/oxr8df96tWk</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -1578,7 +1582,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>• tf2_tools Tutorial: https://docs.ros.org/en/humble/Tutorials/Intermediate/Tf2/Introduction-To-Tf2.html</t>
+          <t>• URDF Display Launch: https://youtu.be/2ri0Ouc67W0</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -1728,8 +1732,9 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>• Gazebo Simulation with ROS 2: https://www.youtube.com/watch?v=fblmuZkWx64
-• SDF Physics Setup: https://www.youtube.com/watch?v=sM12eL34nZk</t>
+          <t>• Simulate Robot in Gazebo: https://youtu.be/wZV1PoZ4fyk
+• Gazebo Camera View: https://youtu.be/fiRRzJV1YIw
+• Automatic Addison Series: https://www.youtube.com/playlist?list=PLNWNEEf8BvG64FVZT4IdieI1PuYnHkUrt</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1757,7 +1762,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>• Gazebo Building Editor: https://www.youtube.com/watch?v=YpS5M8oJ9fE</t>
+          <t>• Gazebo Camera Guide: https://youtu.be/fiRRzJV1YIw</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -1787,7 +1792,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>• Gazebo Sensors - LiDAR &amp; Camera: https://www.youtube.com/watch?v=W3sY4mG2h0A</t>
+          <t>• Simulate Mobile Robot: https://youtu.be/wZV1PoZ4fyk</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1846,7 +1851,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>• Gazebo Topics &amp; Services: https://gazebosim.org/docs</t>
+          <t>• Gazebo Simulation Setup: https://youtu.be/wZV1PoZ4fyk</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">

</xml_diff>

<commit_message>
feat(curriculum): integrate ordered Nav2, SLAM, perception and path planning tutorials for Week 4, 5, and 6
</commit_message>
<xml_diff>
--- a/Apex_Autonomous_7Week_Plan.xlsx
+++ b/Apex_Autonomous_7Week_Plan.xlsx
@@ -2002,8 +2002,10 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>• Driving in Gazebo &amp; RViz View: https://www.youtube.com/watch?v=3iXk5hY5M7g
-• Teleop Twist Keyboard: https://www.youtube.com/watch?v=8qO5sF1Y1c4</t>
+          <t>• Driving in Gazebo &amp; RViz: https://www.youtube.com/watch?v=3iXk5hY5M7g
+• Teleop Twist: https://www.youtube.com/watch?v=8qO5sF1Y1c4
+• Sensor Streaming: https://www.youtube.com/watch?v=7uV8hG9zM3c
+• Gazebo Camera: https://youtu.be/fiRRzJV1YIw</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -2218,7 +2220,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Focus: Perception Pipeline, Computer Vision &amp; 3D Markers | 4 Active Days + 1 Check-in</t>
+          <t>Focus: Perception Pipeline, Sensor Fusion &amp; SLAM | 4 Active Days + 1 Check-in</t>
         </is>
       </c>
     </row>
@@ -2258,25 +2260,29 @@
       <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Main Session 1
-(Vision &amp; SLAM Concepts)</t>
+(Sensors, Transforms &amp; SLAM)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>• Computer vision fundamentals: RGB to HSV color conversion, thresholding
-• ROS 2 cv_bridge: bridging sensor_msgs/Image with OpenCV cv::Mat
-• 2D/3D SLAM concepts and landmark-based localization overview</t>
+          <t>• Common sensors for Nav2 and REP-105 coordinate transformations
+• Sensor fusion localization with EKF and 2D SLAM environment mapping
+• Nav2 stack installation and overview</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>• OpenCV Color &amp; Contour Detection: https://www.youtube.com/watch?v=1_RYMm8L5zQ
-• 2D SLAM with SLAM Toolbox: https://www.youtube.com/watch?v=ZaiA3hW43RE</t>
+          <t>• 1. Common Sensors: https://youtu.be/VSzkBNJegS4
+• 2. Coordinate Transforms: https://youtu.be/eDyHFa1LmpQ
+• 3. Sensor Fusion &amp; Localization: https://youtu.be/XOQTF38lmtE
+• 4. SLAM Mapping: https://youtu.be/VoX5AwTfHuQ
+• 5. Install Nav2: https://youtu.be/gyskLlvX3oI
+• Sensor Fusion Playlist: https://youtube.com/playlist?list=PLn8PRpmsu08ryYoBpEKzoMOveSTyS-h4a&amp;si=B75o2uHrgnkkt5sC</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Study OpenCV color masking and cv_bridge documentation.</t>
+          <t>Study sensors, transforms, and sensor fusion playlist.</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2336,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>• ROS 2 Image Processing with cv_bridge: https://www.youtube.com/watch?v=kYvVqT7C4eY</t>
+          <t>• ROS 2 Image Processing: https://youtu.be/VSzkBNJegS4</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -2528,25 +2534,28 @@
       <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Main Session 1
-(Nav2 &amp; Pure Pursuit Theory)</t>
+(Planning, Nav2 &amp; Control Theory)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>• Nav2 architecture: Costmaps (Global/Local), Planners, and Controllers
-• Pure Pursuit geometry: lookahead distance L, heading error alpha
-• Curvature calculation: kappa = 2*sin(alpha)/L and angular velocity w = kappa * v</t>
+          <t>• Path planning algorithms (A* &amp; RRT) and Nav2 navigation stack
+• Nav2 Simple Commander API in Python
+• Autonomous docking using AprilTags and Pure Pursuit curvature math</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>• Nav2 Overview &amp; Path Planning: https://www.youtube.com/watch?v=jso-I_Pau2o
-• Pure Pursuit Algorithm Explained: https://www.youtube.com/watch?v=u3qBqF39158</t>
+          <t>• 1. Path Planning (A* &amp; RRT): https://youtu.be/QR3U1dgc5RE
+• 2. Autonomous Nav using ROS 2: https://youtu.be/YzTMROP4qos
+• 3. Simple Commander API: https://youtu.be/gKoXrrj2klg
+• 4. AprilTags Docking: https://youtu.be/tFE75bP-ASo
+• Series Playlist: https://www.youtube.com/playlist?list=PLNWNEEf8BvG64FVZT4IdieI1PuYnHkUrt</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Study Pure Pursuit mathematical derivation and parameters.</t>
+          <t>Study path planning theory, commander API, and Pure Pursuit formulas.</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2578,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>• Autonomous Driving Path Tracking: https://www.youtube.com/watch?v=4dJ6Qn_y0tE</t>
+          <t>• Autonomous Driving Path Tracking: https://youtu.be/YzTMROP4qos</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -2599,7 +2608,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>• Writing a Path Follower in ROS 2: https://www.youtube.com/watch?v=4dJ6Qn_y0tE</t>
+          <t>• Writing a Path Follower in ROS 2: https://youtu.be/gKoXrrj2klg</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">

</xml_diff>